<commit_message>
Plantilla de Excel propia de la app (sin Hub, sin Pauta ni Asignado a) y exportar con las mismas columnas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QtS8C8GC6PUTqNPYTJiSZE
</commit_message>
<xml_diff>
--- a/calendario/plantillas/Plantilla_Calendario_Contenidos.xlsx
+++ b/calendario/plantillas/Plantilla_Calendario_Contenidos.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -497,9 +497,10 @@
     <col width="40" customWidth="1" min="14" max="14"/>
     <col width="45" customWidth="1" min="15" max="15"/>
     <col width="45" customWidth="1" min="16" max="16"/>
-    <col width="32" customWidth="1" min="17" max="17"/>
-    <col width="30" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -585,32 +586,22 @@
       </c>
       <c r="Q1" s="4" t="inlineStr">
         <is>
-          <t>Pauta</t>
+          <t>Link pieza terminada</t>
         </is>
       </c>
       <c r="R1" s="4" t="inlineStr">
         <is>
-          <t>Link pieza terminada</t>
+          <t>Link material de referencia</t>
         </is>
       </c>
       <c r="S1" s="4" t="inlineStr">
         <is>
-          <t>Link material de referencia</t>
+          <t>Notas internas</t>
         </is>
       </c>
       <c r="T1" s="4" t="inlineStr">
         <is>
-          <t>Notas internas</t>
-        </is>
-      </c>
-      <c r="U1" s="7" t="inlineStr">
-        <is>
-          <t>Asignado a</t>
-        </is>
-      </c>
-      <c r="V1" s="4" t="inlineStr">
-        <is>
-          <t>Pilar / fase (referencia interna, NO se sube al hub)</t>
+          <t>Pilar / fase (referencia interna, NO se sube a la app)</t>
         </is>
       </c>
     </row>
@@ -690,19 +681,14 @@
           <t>Ej: Plano 1: producto entero sobre mesa de madera clara. Plano 2: primer plano de la mano abriendo el envase. Plano 3: producto servido, luz cálida.</t>
         </is>
       </c>
-      <c r="Q2" s="5" t="inlineStr">
-        <is>
-          <t>Solo orgánico</t>
-        </is>
-      </c>
+      <c r="Q2" s="5" t="inlineStr"/>
       <c r="R2" s="5" t="inlineStr"/>
-      <c r="S2" s="5" t="inlineStr"/>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>Ejemplo de fila — borrala y cargá tus propios contenidos.</t>
+        </is>
+      </c>
       <c r="T2" s="5" t="inlineStr">
-        <is>
-          <t>Ejemplo de fila — borrala y cargá tus propios contenidos.</t>
-        </is>
-      </c>
-      <c r="V2" s="5" t="inlineStr">
         <is>
           <t>Septiembre · Ejemplo</t>
         </is>
@@ -719,7 +705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A53"/>
+  <dimension ref="A1:A49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -728,7 +714,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PLANTILLA BASE — Carga de contenidos al COSMART Marketing Hub</t>
+          <t>PLANTILLA BASE — Carga de contenidos al Calendario de contenidos</t>
         </is>
       </c>
     </row>
@@ -738,7 +724,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Esta hoja ('Contenidos') tiene una columna por cada campo del formulario 'Nuevo contenido' del hub.</t>
+          <t>Esta hoja ('Contenidos') tiene una columna por cada campo del formulario 'Nuevo contenido' de la app.</t>
         </is>
       </c>
     </row>
@@ -762,7 +748,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>1. En el hub, sección Contenidos → botón 'Importar Excel'.</t>
+          <t>1. En la app, sección Contenidos → botón 'Importar Excel'.</t>
         </is>
       </c>
     </row>
@@ -776,7 +762,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>3. El hub identifica cada fila por Título + Cuenta:</t>
+          <t>3. La app identifica cada fila por Título + Cuenta:</t>
         </is>
       </c>
     </row>
@@ -849,7 +835,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>• Cuenta (el handle configurado en el hub, ej: minamiworldok)</t>
+          <t>• Cuenta (el handle que cargaste en Mis cuentas, ej: tumarca)</t>
         </is>
       </c>
     </row>
@@ -868,16 +854,16 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>ASIGNAR EL CONTENIDO A ALGUIEN (opcional)</t>
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>CAMPOS QUE ACEPTAN VARIOS VALORES (separar con coma dentro de la misma celda)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>• Columna 'Asignado a': escribí el nombre o el email de a quién se lo querés asignar -- tiene que ser el contacto del cliente o alguien del equipo ya agregado a este cliente en el hub. Si no coincide con nadie, se sube sin asignar (no da error).</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Plataformas, Ubicación, Formato, Dimensiones — ej: 'Instagram, TikTok' o 'Feed, Story'.</t>
         </is>
       </c>
     </row>
@@ -887,166 +873,143 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>CAMPOS QUE ACEPTAN VARIOS VALORES (separar con coma dentro de la misma celda)</t>
+          <t>COPY vs. TEXTO EN PANTALLA — son dos cosas distintas, no las mezcles</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Plataformas, Ubicación, Formato, Dimensiones — ej: 'Instagram, TikTok' o 'Feed, Story'.</t>
+          <t>• Copy: el texto de la descripción/caption del posteo (lo que se lee debajo, en el feed).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>• Texto en pantalla: el texto que aparece escrito DENTRO de la pieza (imagen o video).</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>COPY vs. TEXTO EN PANTALLA — son dos cosas distintas, no las mezcles</t>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>• Prompt sugerido para IA: si esa pieza se va a generar con inteligencia artificial, el prompt sugerido para armarla (opcional).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>• Copy: el texto de la descripción/caption del posteo (lo que se lee debajo, en el feed).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>• Texto en pantalla: el texto que aparece escrito DENTRO de la pieza (imagen o video).</t>
-        </is>
-      </c>
-    </row>
+          <t>• Sugerencia de pieza creativa: cómo se imagina la pieza visualmente -- descripción de la imagen, o secuencia de escenas/planos si es un video (distinto del prompt de IA de arriba, es para guiar a quien diseña/filma, se use o no IA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>• Prompt sugerido para IA: si esa pieza se va a generar con inteligencia artificial, el prompt sugerido para armarla (opcional).</t>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>GUION Y TELEPROMPTER (opcional)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>• Sugerencia de pieza creativa: cómo se imagina la pieza visualmente -- descripción de la imagen, o secuencia de escenas/planos si es un video (distinto del prompt de IA de arriba, es para guiar a quien diseña/filma, se use o no IA).</t>
-        </is>
-      </c>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>• Columna 'Guion': el texto completo para leer mientras se graba la pieza. Adentro de la app, cada guion tiene un botón para abrir el teleprompter, que lo muestra a pantalla completa (fondo negro, letras blancas, auto-scroll).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>GUION Y TELEPROMPTER (opcional)</t>
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>VALORES VÁLIDOS POR COLUMNA</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>• Columna 'Guion': el texto completo para leer mientras se graba la pieza. Adentro del hub, cada contenido tiene un botón '📺 Abrir teleprompter' que lo muestra a pantalla completa (fondo negro, letras blancas, auto-scroll).</t>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Estado: Idea, En proceso, En revisión, Aprobado, Programado, Publicado</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Plataformas: Instagram, Facebook, LinkedIn, Twitter / X, TikTok, YouTube, Sitio Web, Blog</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>VALORES VÁLIDOS POR COLUMNA</t>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Ubicación según plataforma — Instagram/Facebook: Feed, Story, Reel, Carrusel · TikTok: Feed, Story · YouTube: Feed, Shorts · LinkedIn/Twitter: Feed</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Estado: Idea, En proceso, En revisión, Aprobado, Programado, Publicado</t>
+          <t>Formato según plataforma — Instagram: Imagen, Video, Reel, Carrusel, Story, GIF · TikTok: Video · YouTube: Video · LinkedIn: Imagen, Video, Carrusel, Documento</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Plataformas: Instagram, Facebook, LinkedIn, Twitter / X, TikTok, YouTube, Sitio Web, Blog</t>
+          <t>Dimensiones: 1:1, 4:5, 9:16, 16:9, 1.91:1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Ubicación según plataforma — Instagram/Facebook: Feed, Story, Reel, Carrusel · TikTok: Feed, Story · YouTube: Feed, Shorts · LinkedIn/Twitter: Feed</t>
+          <t>Eje de comunicación: Institucional, Entretenimiento, Comercial, Interacción, Educativo, Inspiracional</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Formato según plataforma — Instagram: Imagen, Video, Reel, Carrusel, Story, GIF · TikTok: Video · YouTube: Video · LinkedIn: Imagen, Video, Carrusel, Documento</t>
+          <t>Tipo de contenido: Informativo, Promocional, Sorteo, Viral, Evento, Celebración, Tutorial</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Dimensiones: 1:1, 4:5, 9:16, 16:9, 1.91:1</t>
+          <t>Objetivo: Notoriedad, Engagement, Alcance, Conversión, Tráfico</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Eje de comunicación: Institucional, Entretenimiento, Comercial, Interacción, Educativo, Inspiracional</t>
-        </is>
-      </c>
+      <c r="A45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Tipo de contenido: Informativo, Promocional, Sorteo, Viral, Evento, Celebración, Tutorial</t>
+          <t>Fecha de publicación: formato AAAA-MM-DD (ej: 2026-08-15). Si Excel la formatea como fecha, funciona igual.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: Notoriedad, Engagement, Alcance, Conversión, Tráfico</t>
-        </is>
-      </c>
+      <c r="A47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Pauta: Solo orgánico, Sí – Dark post, Sí – Dark + orgánico</t>
+          <t>La última columna ('Pilar / fase') es solo para planificación estratégica interna: no es un campo de la app y se descarta al importar.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Fecha de publicación: formato AAAA-MM-DD (ej: 2026-08-15). Si Excel la formatea como fecha, funciona igual.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>La última columna ('Pilar / fase') es solo para planificación estratégica interna: no es un campo del hub y se descarta al importar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>Los campos que no están en esta plantilla (comentarios, archivos adjuntos) se completan después, ya adentro del hub.</t>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Los campos que no están en esta plantilla (comentarios, archivos adjuntos) se completan después, ya adentro de la app.</t>
         </is>
       </c>
     </row>

</xml_diff>